<commit_message>
spec: drop whole-scenario 'Repeat 1~N for M times' steps (handled by --iterations)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -2083,8 +2083,7 @@
 3. Restore connectivity
 4. Verify DNS traffic steered after recovery
 5. Change steering mode during FailClose active
-6. Verify correct enforcement after mode change completes
-7. Repeat 1~6 for 20 times</t>
+6. Verify correct enforcement after mode change completes</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -2152,8 +2151,7 @@
 2. Monitor client status API call rate from endpoint
 3. Verify client implements backoff/throttling
 4. Verify client config downloads still succeed during status storm
-5. Monitor backend response times
-6. Repeat 1~5 for 20 times</t>
+5. Monitor backend response times</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2221,8 +2219,7 @@
 2. Put device to Modern Standby
 3. Wake device and verify client status updates correctly
 4. Trigger auto-upgrade while device in AOAC mode
-5. Verify enrollment survives upgrade + wake cycle
-6. Repeat 1~5 for 20 times</t>
+5. Verify enrollment survives upgrade + wake cycle</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2290,8 +2287,7 @@
 2. Block gateway IP at firewall
 3. Reboot device
 4. After boot, verify all non-exempt traffic is blocked
-5. Unblock gateway and verify tunnel re-establishes
-6. Repeat 1~5 for 20 times</t>
+5. Unblock gateway and verify tunnel re-establishes</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2360,8 +2356,7 @@
 3. Verify uninstall blocked
 4. Send IOCTL commands to driver attempting disable
 5. Verify driver rejects unauthorized IOCTL
-6. Verify service remains running and protected
-7. Repeat 1~6 for 20 times</t>
+6. Verify service remains running and protected</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2429,8 +2424,7 @@
 2. Generate large DNS TCP responses (&gt;512 bytes, fragmented)
 3. Verify packets not dropped or corrupted
 4. Monitor for BSOD/crash
-5. Verify DNS resolution latency stays under threshold
-6. Repeat 1~5 for 20 times</t>
+5. Verify DNS resolution latency stays under threshold</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2499,8 +2493,7 @@
 3. Verify packets not dropped or corrupted
 4. Run DNS load test on Citrix/VDI with 50+ concurrent sessions
 5. Monitor for BSOD/crash
-6. Verify DNS resolution latency stays under threshold
-7. Repeat 1~6 for 20 times</t>
+6. Verify DNS resolution latency stays under threshold</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2568,8 +2561,7 @@
 2. Start auto-upgrade.
 3. Kill msiexec process mid-installation (simulating crash).
 4. Reboot.
-5. Verify UpgradeInProgress registry is eventually cleared and watchdog resumes monitoring.
-6. Repeat 1~5 for 20 times</t>
+5. Verify UpgradeInProgress registry is eventually cleared and watchdog resumes monitoring.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2637,8 +2629,7 @@
 2. Verify client performs GSLB re-evaluation and selects better DP
 3. Block DTLS port
 4. Verify automatic failover to TLS within timeout
-5. Restore DTLS and verify client returns to DTLS
-6. Repeat 1~5 for 20 times</t>
+5. Restore DTLS and verify client returns to DTLS</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2706,8 +2697,7 @@
 2. Restart service and verify recovery from backup
 3. Delete user cert while config encryption enabled
 4. Verify client re-downloads config without crash
-5. Verify client does not remain disabled
-6. Repeat 1~5 for 20 times</t>
+5. Verify client does not remain disabled</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2776,8 +2766,7 @@
 3. Verify upgrade triggers at correct time
 4. Interrupt upgrade mid-MSI (kill msiexec process)
 5. Reboot and verify Legacy Monitor retries and completes upgrade
-6. Verify client not silently removed
-7. Repeat 1~6 for 5 times</t>
+6. Verify client not silently removed</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2846,8 +2835,7 @@
 3. Login User B simultaneously on same machine
 4. Verify User A connections not disrupted
 5. Verify User B gets correct steering config
-6. Logout User A and verify User B tunnel persists
-7. Repeat 1~6 for 20 times</t>
+6. Logout User A and verify User B tunnel persists</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2916,8 +2904,7 @@
 3. Verify enrollment completes without timeout
 4. Test enrollment during Windows Autopilot OOBE
 5. Verify no blank enrollment window from concurrent webview2
-6. Verify enrollment on subsequent Citrix sessions
-7. Repeat 1~6 for 20 times</t>
+6. Verify enrollment on subsequent Citrix sessions</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2985,8 +2972,7 @@
 2. Verify only that app's traffic bypasses tunnel
 3. Generate traffic from other apps
 4. Verify other apps still steered through tunnel
-5. Change steering config and verify cert-pinned exception still scoped correctly
-6. Repeat 1~5 for 20 times</t>
+5. Change steering config and verify cert-pinned exception still scoped correctly</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -3053,8 +3039,7 @@
           <t>1. Configure client with FailClose + All Traffic steering
 2. Repeatedly stop/start service via net stop stAgentSvc
 3. Toggle sleep/wake and network adapters concurrently
-4. Monitor for crash dumps in C:\dump
-5. Repeat 1~4 for 20 times</t>
+4. Monitor for crash dumps in C:\dump</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -3123,8 +3108,7 @@
 3. Verify steering disabled per on-prem policy
 4. Switch to off-prem network (different egress IP)
 5. Verify client detects transition and reconnects tunnel
-6. Verify steering re-enabled within 30s
-7. Repeat 1~6 for 20 times</t>
+6. Verify steering re-enabled within 30s</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -3191,8 +3175,7 @@
           <t>1. Enable self-protection and watchdog.
 2. Trigger auto-upgrade from R135.
 3. Force reboot during CA_RollbackInstallDriver phase.
-4. Boot and verify client presence.
-5. Repeat 1~4 for 5 times</t>
+4. Boot and verify client presence.</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -3260,8 +3243,7 @@
 2. Establish tunnel.
 3. Enter S0 standby (close lid).
 4. Wake repeatedly under varying load.
-5. Monitor for crash dumps and service recovery.
-6. Repeat 1~5 for 20 times</t>
+5. Monitor for crash dumps and service recovery.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -3328,8 +3310,7 @@
           <t>1. Enable watchdog FF via tenant config push.
 2. Verify stWatchdog service is running.
 3. Disable watchdog FF via tenant config push.
-4. Verify stWatchdog service is stopped and removed from SCM.
-5. Repeat 1~4 for 20 times</t>
+4. Verify stWatchdog service is stopped and removed from SCM.</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -3396,8 +3377,7 @@
           <t>1. Enable watchdog FF.
 2. Suspend stAgentSvc process immediately after SCM marks it START_PENDING.
 3. Wait &gt;5 minutes.
-4. Observe whether watchdog takes corrective action or remains dormant.
-5. Repeat 1~4 for 20 times</t>
+4. Observe whether watchdog takes corrective action or remains dormant.</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -3465,8 +3445,7 @@
 2. Generate heavy SMB traffic (file shares, DFS)
 3. Monitor domain controller CPU utilization
 4. Verify NSClient does not amplify SMB connections
-5. Monitor client crash under massive connection load
-6. Repeat 1~5 for 20 times</t>
+5. Monitor client crash under massive connection load</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -3533,8 +3512,7 @@
           <t>1. Deploy NSClient on multi-session Citrix/AVD with FailClose enabled
 2. Login first user and verify tunnel
 3. Login second user whose AppData is not yet initialized
-4. Verify first user session is not disrupted
-5. Repeat 1~4 for 20 times</t>
+4. Verify first user session is not disrupted</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -3601,8 +3579,7 @@
           <t>1. Install NSClient in IDP+peruserconfig mode on multi-session AVD
 2. First user logs in and completes IDP enrollment
 3. Second user logs in
-4. Verify second user gets IDP authentication prompt (not silent UPN enrollment)
-5. Repeat 1~4 for 20 times</t>
+4. Verify second user gets IDP authentication prompt (not silent UPN enrollment)</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -3670,8 +3647,7 @@
 2. Trigger auto-upgrade.
 3. Force reboot/power-off during MSI installation phase.
 4. Boot and trigger another auto-upgrade.
-5. Verify binary version matches registered version.
-6. Repeat 1~5 for 5 times</t>
+5. Verify binary version matches registered version.</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -3739,8 +3715,7 @@
 2. Enable secure enrollment + fail-close.
 3. Have 5+ users log in simultaneously.
 4. Introduce tunnel delay (17+ seconds).
-5. Verify traffic steering.
-6. Repeat 1~5 for 20 times</t>
+5. Verify traffic steering.</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -3808,8 +3783,7 @@
 2. Do admin disable then enable.
 3. Change network.
 4. Attempt to access blocked sites via IPv6 (configure hosts file with IPv6 addresses).
-5. Verify traffic blocked.
-6. Repeat 1~5 for 20 times</t>
+5. Verify traffic blocked.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -3876,8 +3850,7 @@
           <t>1. Enable fail-close and reset_with_overlapped_io FF.
 2. Run client under continuous traffic.
 3. Perform network switches repeatedly for hours.
-4. Monitor for crash dumps.
-5. Repeat 1~4 for 20 times</t>
+4. Monitor for crash dumps.</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -3943,8 +3916,7 @@
         <is>
           <t>1. Install 32-bit NSClient with secure enrollment (tokens in WOW6432Node).
 2. Trigger auto-upgrade to 64-bit MSI.
-3. After upgrade verify enrollment tokens exist under HKLM\Software\Netskope\SecureToken.
-4. Repeat 1~3 for 5 times</t>
+3. After upgrade verify enrollment tokens exist under HKLM\Software\Netskope\SecureToken.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -4012,8 +3984,7 @@
 2. Verify IPv6 traffic correctly steered through tunnel
 3. Add IPv6 local-link exception
 4. Verify local-link IPv6 traffic bypassed
-5. Run throughput test over IPv6 and compare with IPv4 baseline
-6. Repeat 1~5 for 20 times</t>
+5. Run throughput test over IPv6 and compare with IPv4 baseline</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
@@ -4080,8 +4051,7 @@
           <t>1. Enable AOAC, self-protection, fail-close on Windows device.
 2. Put device into hibernate/S0 sleep.
 3. Trigger auto-upgrade immediately after wake.
-4. Monitor SCM callback timing and MSI completion.
-5. Repeat 1~4 for 20 times</t>
+4. Monitor SCM callback timing and MSI completion.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -4148,8 +4118,7 @@
           <t>1. Enable AOAC + fail-close on Windows.
 2. Run under system stress (many apps, high memory).
 3. Cycle sleep/wake repeatedly (20+ times).
-4. Monitor for error 1453 and tunnel disconnection.
-5. Repeat 1~4 for 20 times</t>
+4. Monitor for error 1453 and tunnel disconnection.</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -4216,8 +4185,7 @@
           <t>1. Configure cloud steering mode with domain exceptions.
 2. Switch steering config to web mode (different exception list).
 3. Verify exception list downloads successfully before tunnel disconnects.
-4. Confirm bypassed domains remain accessible.
-5. Repeat 1~4 for 20 times</t>
+4. Confirm bypassed domains remain accessible.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -4284,8 +4252,7 @@
           <t>1. Enable secure config encryption on tenant.
 2. Enable watchdog FF.
 3. Reboot machine.
-4. Verify stWatchdog service starts within 90 seconds of boot.
-5. Repeat 1~4 for 20 times</t>
+4. Verify stWatchdog service starts within 90 seconds of boot.</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -4483,8 +4450,7 @@
         <is>
           <t>1. Configure scheduled upgrade with daily frequency and specific time
 2. Install client and wait for scheduled upgrade window to pass
-3. Verify client remains functional and does not enter hung/disabled state
-4. Repeat 1~3 for 5 times</t>
+3. Verify client remains functional and does not enter hung/disabled state</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -4551,8 +4517,7 @@
           <t>1. Configure FailClose with dynamic steering disabled
 2. Reboot Windows device
 3. At login screen, attempt Self-Service Password Reset (SSPR)
-4. Verify SSPR traffic (passwordreset.microsoftonline.com) is not blocked
-5. Repeat 1~4 for 20 times</t>
+4. Verify SSPR traffic (passwordreset.microsoftonline.com) is not blocked</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
@@ -4619,8 +4584,7 @@
           <t>1. Enable Secure Config validation on tenant
 2. Deploy NSClient and verify initial config download
 3. Trigger feature flag update from admin
-4. Verify subsequent steering config downloads succeed (no 405 error)
-5. Repeat 1~4 for 20 times</t>
+4. Verify subsequent steering config downloads succeed (no 405 error)</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
@@ -4687,8 +4651,7 @@
           <t>1. Install NSClient older version
 2. Delete Logs folder under %appdata%\Netskope\stagent
 3. Trigger auto-upgrade via config push
-4. Verify upgrade completes
-5. Repeat 1~4 for 5 times</t>
+4. Verify upgrade completes</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: drop 'consistent results across all N repetitions' pass-criteria clause (iterations-handled)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -2088,7 +2088,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>DNS traffic steered correctly after FailClose recovery; steering mode change during FailClose does not leave inconsistent state; consistent results across all 20 repetitions with no degradation</t>
+          <t>DNS traffic steered correctly after FailClose recovery; steering mode change during FailClose does not leave inconsistent state</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Client throttles status updates to &lt;1 per 60s; config downloads succeed within 30s during storm; no cascading failure; consistent results across all 20 repetitions with no degradation</t>
+          <t>Client throttles status updates to &lt;1 per 60s; config downloads succeed within 30s during storm; no cascading failure</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Client remains enabled with correct status after AOAC wake; upgrade completes without enrollment loss on AOAC device; consistent results across all 20 repetitions with no degradation</t>
+          <t>Client remains enabled with correct status after AOAC wake; upgrade completes without enrollment loss on AOAC device</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>All non-exempt traffic blocked immediately after boot even when gateway is unreachable; tunnel recovers when gateway accessible again; consistent results across all 20 repetitions with no degradation</t>
+          <t>All non-exempt traffic blocked immediately after boot even when gateway is unreachable; tunnel recovers when gateway accessible again</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>All third-party uninstall attempts blocked; unauthorized IOCTL commands rejected; client remains enabled and protected; consistent results across all 20 repetitions with no degradation</t>
+          <t>All third-party uninstall attempts blocked; unauthorized IOCTL commands rejected; client remains enabled and protected</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>No packet drops for large DNS TCP; no BSOD; DNS latency &lt;100ms under 50-session load on VDI; consistent results across all 20 repetitions with no degradation</t>
+          <t>No packet drops for large DNS TCP; no BSOD; DNS latency &lt;100ms under 50-session load on VDI</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>No packet drops for large DNS TCP; no BSOD; DNS latency &lt;100ms under 50-session load on VDI; consistent results across all 20 repetitions with no degradation</t>
+          <t>No packet drops for large DNS TCP; no BSOD; DNS latency &lt;100ms under 50-session load on VDI</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>After reboot, UpgradeMonitorThread detects aborted upgrade, retries MSI, and clears UpgradeInProgress within 3 hours; consistent results across all 20 repetitions with no degradation</t>
+          <t>After reboot, UpgradeMonitorThread detects aborted upgrade, retries MSI, and clears UpgradeInProgress within 3 hours</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Client selects optimal DP via GSLB; DTLS-to-TLS failover completes within 30s; client returns to DTLS when available; consistent results across all 20 repetitions with no degradation</t>
+          <t>Client selects optimal DP via GSLB; DTLS-to-TLS failover completes within 30s; client returns to DTLS when available</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Client recovers from corrupted config via backup mechanism; cert deletion does not crash service; client re-enrolls automatically; consistent results across all 20 repetitions with no degradation</t>
+          <t>Client recovers from corrupted config via backup mechanism; cert deletion does not crash service; client re-enrolls automatically</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Upgrade triggers on scheduled day; interrupted upgrade recovered by Legacy Monitor; client never left in removed state; consistent results across all 5 repetitions with no degradation</t>
+          <t>Upgrade triggers on scheduled day; interrupted upgrade recovered by Legacy Monitor; client never left in removed state</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>No traffic disruption for existing sessions during concurrent logon; each user gets correct steering; logout does not break other sessions; consistent results across all 20 repetitions with no degradation</t>
+          <t>No traffic disruption for existing sessions during concurrent logon; each user gets correct steering; logout does not break other sessions</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>IDP enrollment succeeds on Citrix first login; Autopilot enrollment completes; no blank webview2 windows; consistent results across all 20 repetitions with no degradation</t>
+          <t>IDP enrollment succeeds on Citrix first login; Autopilot enrollment completes; no blank webview2 windows</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Only cert-pinned app traffic bypasses; all other traffic remains steered; config change does not broaden exception scope; consistent results across all 20 repetitions with no degradation</t>
+          <t>Only cert-pinned app traffic bypasses; all other traffic remains steered; config change does not broaden exception scope</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>No stAgentSvc crash dumps generated across 50 service stop/start cycles with concurrent network events; consistent results across all 20 repetitions with no degradation</t>
+          <t>No stAgentSvc crash dumps generated across 50 service stop/start cycles with concurrent network events</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>On-prem correctly detected via egress IP; off-prem transition triggers tunnel reconnect within 30s; steering resumes; consistent results across all 20 repetitions with no degradation</t>
+          <t>On-prem correctly detected via egress IP; off-prem transition triggers tunnel reconnect within 30s; steering resumes</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>After reboot, installation monitor service detects incomplete upgrade and retries. Client is present and functional; consistent results across all 5 repetitions with no degradation</t>
+          <t>After reboot, installation monitor service detects incomplete upgrade and retries. Client is present and functional</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Service never crashes on wake. Write-packet thread waits for driver initialization. No null pointer access; consistent results across all 20 repetitions with no degradation</t>
+          <t>Service never crashes on wake. Write-packet thread waits for driver initialization. No null pointer access</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>stWatchdog service no longer appears in services.msc; UpgradeInProgress registry absent; no orphan stAgentSvcMon.exe on disk; consistent results across all 20 repetitions with no degradation</t>
+          <t>stWatchdog service no longer appears in services.msc; UpgradeInProgress registry absent; no orphan stAgentSvcMon.exe on disk</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Watchdog eventually force-kills and restarts the hung service, or escalates via log error after N cycles; consistent results across all 20 repetitions with no degradation</t>
+          <t>Watchdog eventually force-kills and restarts the hung service, or escalates via log error after N cycles</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>DC CPU stays below 80% during SMB operations with NSClient; no connection amplification; no client crash; consistent results across all 20 repetitions with no degradation</t>
+          <t>DC CPU stays below 80% during SMB operations with NSClient; no connection amplification; no client crash</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>New user session failure to read nsuser.conf does not trigger FailClose for existing active sessions; consistent results across all 20 repetitions with no degradation</t>
+          <t>New user session failure to read nsuser.conf does not trigger FailClose for existing active sessions</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>Second and subsequent users must complete IDP authentication before enrollment; no silent UPN bypass; consistent results across all 20 repetitions with no degradation</t>
+          <t>Second and subsequent users must complete IDP authentication before enrollment; no silent UPN bypass</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>After recovery, stAgentSvc runs the new version. No version mismatch between appinfo.log and running binary; consistent results across all 5 repetitions with no degradation</t>
+          <t>After recovery, stAgentSvc runs the new version. No version mismatch between appinfo.log and running binary</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>nsFilterDevice config reloads correctly regardless of multi-user logon timing. All traffic steered through inner tunnel; consistent results across all 20 repetitions with no degradation</t>
+          <t>nsFilterDevice config reloads correctly regardless of multi-user logon timing. All traffic steered through inner tunnel</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>IPv6 traffic without hostname is blocked (not bypassed). m_forceTearDown resets correctly after admin enable; consistent results across all 20 repetitions with no degradation</t>
+          <t>IPv6 traffic without hostname is blocked (not bypassed). m_forceTearDown resets correctly after admin enable</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>No service crash during extended network switching. Overlapped IO prevents indefinite DeviceIoControl blocking; consistent results across all 20 repetitions with no degradation</t>
+          <t>No service crash during extended network switching. Overlapped IO prevents indefinite DeviceIoControl blocking</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>AuthenticationToken and EncryptionToken data values exist and match pre-upgrade values; device does not require re-enrollment; consistent results across all 5 repetitions with no degradation</t>
+          <t>AuthenticationToken and EncryptionToken data values exist and match pre-upgrade values; device does not require re-enrollment</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -3989,7 +3989,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>IPv6 traffic correctly steered; local-link exceptions honored; IPv6 throughput within 20% of IPv4 baseline; consistent results across all 20 repetitions with no degradation</t>
+          <t>IPv6 traffic correctly steered; local-link exceptions honored; IPv6 throughput within 20% of IPv4 baseline</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Upgrade completes within SCM timeout. Service stop token is accepted. No MSI rollback occurs; consistent results across all 20 repetitions with no degradation</t>
+          <t>Upgrade completes within SCM timeout. Service stop token is accepted. No MSI rollback occurs</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>On quota error, stadrv restarts automatically. Tunnel reconnects without manual intervention. No persistent fail-close state; consistent results across all 20 repetitions with no degradation</t>
+          <t>On quota error, stadrv restarts automatically. Tunnel reconnects without manual intervention. No persistent fail-close state</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>All mandatory config downloads complete before tunnel teardown. No traffic mode enforcement without valid exception list; consistent results across all 20 repetitions with no degradation</t>
+          <t>All mandatory config downloads complete before tunnel teardown. No traffic mode enforcement without valid exception list</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>stWatchdog service state is SERVICE_RUNNING; nswatchdog_log shows successful startup entry; consistent results across all 20 repetitions with no degradation</t>
+          <t>stWatchdog service state is SERVICE_RUNNING; nswatchdog_log shows successful startup entry</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>Client remains enabled and functional; scheduled upgrade triggers correctly without hanging; consistent results across all 5 repetitions with no degradation</t>
+          <t>Client remains enabled and functional; scheduled upgrade triggers correctly without hanging</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>SSPR workflow completes at Windows login screen despite FailClose being configured; consistent results across all 20 repetitions with no degradation</t>
+          <t>SSPR workflow completes at Windows login screen despite FailClose being configured</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>Steering config downloads successfully after feature flag changes; no 405 errors in client logs; consistent results across all 20 repetitions with no degradation</t>
+          <t>Steering config downloads successfully after feature flag changes; no 405 errors in client logs</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>Upgrade completes successfully; installer creates missing Logs folder before launching msiexec; consistent results across all 5 repetitions with no degradation</t>
+          <t>Upgrade completes successfully; installer creates missing Logs folder before launching msiexec</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: rewrite STRESS-05 (HTTPS flood + crash/watchdog-restart + sc restart, 61s)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -666,19 +666,18 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1. Verify stAgentSvc and stAgentSvcWD are both running
-2. taskkill /F /IM stAgentSvc.exe (force kill — simulates crash)
-3. Wait up to 60 seconds (watchdog check interval)
-4. Verify stAgentSvcWD detects abnormal stop (Win32ExitCode != ERROR_SUCCESS)
-5. Verify stAgentSvc is restarted automatically
-6. Verify tunnel re-establishes after restart
-7. Repeat: kill during active traffic — verify no permanent state corruption
-8. Test edge case: kill stAgentSvc during upgrade (UpgradeInProgress=1 in registry) — watchdog should NOT restart</t>
+          <t>1. Verify stAgentSvc and stAgentSvcMon are both running
+2. Verify tunnel is established
+3. Generate HTTPS flooding by 600 conn in 30 threads
+4. taskkill /F /IM stAgentSvc.exe (force kill — simulates crash)
+5. Verify stAgentSvc is restarted automatically and tunnel re-establishes within 60s
+6. Generate HTTPS flooding by 600 conn in 30 threads
+7. restart stAgentSvc (sc stop stagentsvc and sc start stagentsvc)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Watchdog restarts service within 60-90s. Tunnel recovers. No restart during upgrade. No permanent state corruption after crash+restart.</t>
+          <t>Watchdog restarts service within 61s. Tunnel recovers. No restart during upgrade. No permanent state corruption after crash+restart.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: STRESS-07 step-7 = deliberate fail-open on service crash (both copies)
Same change as nsclient_test_base: crash window fail-open is the driver's
auto-teardown design (measured 3/3 on develop-141); hard assertion moves
to post-watchdog re-engagement while still fenced.

Agent: git33-kimi-k3
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -736,19 +736,19 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Enable FailClose in client configuration
+          <t>1. Enable FailClose in client configuration
 2. Establish tunnel — verify normal traffic flows
-3. Simulate gateway unreachable (block gateway IP/hostname at firewall + hosts; block BOTH primary and backup gateway, and chase GSLB POP switches after the client restart, or the client reconnects to an unblocked POP and never fail-closes)
+3. Simulate gateway unreachable (block gateway IP at firewall/hosts)
 4. Verify: all user traffic is blocked (cannot browse, cannot reach any external site)
-5. (OPTIONAL — SKIPPED: needs a captive-portal-capable WiFi environment, which no current lane VM has; the client-side WiFi toggle helper does not exist either. Track separately, do not gate this case on it.) Verify: captive portal detection triggers if connecting to new WiFi with portal
-6. Restore gateway access — verify tunnel reconnects AND traffic unblocks
-7. Test edge case: service crash with FailClose ON — verify traffic blocks during the crash window, unblocks after watchdog restart
-8. (OPTIONAL — NPA-licensed tenants only. Auto-detect with nsdiag -n and skip when it reports NPA status Disabled or gateway IP N/A, same pattern as STRESS-03.) Test edge case: FailClose + NPA-only tunnel (ENG-1012026 pattern) — verify cert-pinned apps are also blocked</t>
+5. (OPTIONAL — requires a captive-portal-capable WiFi environment, not available on current lane VMs; non-blocking) Verify: captive portal detection triggers if connecting to new WiFi with portal
+6. Restore gateway access — verify tunnel reconnects AND traffic unblocks WITHOUT a client restart (a recovery needing a restart hides the stuck-blocking bug)
+7. Test edge case: service crash with FailClose ON. EXPECTED fail-open: killing stAgentSvc tears down the WFP blocking (driver auto-teardown on device-handle close — availability over security for the agent's own crash), so traffic FLOWS during the crash window. The hard assertion is AFTER the watchdog restart: with the gateway still blocked, FailClose must RE-ENGAGE (traffic blocked again); then restore gateway access — traffic unblocks
+8. (OPTIONAL — NPA-licensed tenants only; auto-detect via nsdiag -n, skip when NPA status is N/A, mirroring STRESS-03's NPA pattern) Test edge case: FailClose + NPA-only tunnel (ENG-1012026 pattern) — verify cert-pinned apps are also blocked</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">All non-exempt traffic blocked while the gateway is unreachable; tunnel and traffic both recover when the gateway is accessible again, WITHOUT restarting the client (a restart-only recovery is a fail — it hides the stuck-blocking bug). No permanent block state. During the crash window: traffic blocked while the service is down, unblocked after the watchdog restart. Captive portal detection works (only when step 5 is exercised; a skipped run must not report it as passed).</t>
+          <t>All non-exempt traffic blocked while FailClose is engaged (gateway unreachable). Traffic restored after gateway recovery WITHOUT a client restart. No permanent block state. Service crash is a deliberate FAIL-OPEN (driver auto-teardown): traffic flows during the crash window — this is expected, NOT a failure. After the watchdog restarts the service with the gateway still blocked, FailClose must re-engage and block again. Captive portal detection works (OPTIONAL — non-blocking until a captive-portal-capable environment exists). Cert-pinned apps blocked under FailClose + NPA-only tunnel (OPTIONAL — verified only on NPA-licensed tenants, auto-detected via nsdiag -n; skipped when N/A).</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: STRESS-07 step-7 + pass criteria simplified (both copies)
Agent: git33-kimi-k3
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -741,14 +741,14 @@
 3. Simulate gateway unreachable (block gateway IP at firewall/hosts)
 4. Verify: all user traffic is blocked (cannot browse, cannot reach any external site)
 5. (OPTIONAL — requires a captive-portal-capable WiFi environment, not available on current lane VMs; non-blocking) Verify: captive portal detection triggers if connecting to new WiFi with portal
-6. Restore gateway access — verify tunnel reconnects AND traffic unblocks WITHOUT a client restart (a recovery needing a restart hides the stuck-blocking bug)
-7. Test edge case: service crash with FailClose ON. EXPECTED fail-open: killing stAgentSvc tears down the WFP blocking (driver auto-teardown on device-handle close — availability over security for the agent's own crash), so traffic FLOWS during the crash window. The hard assertion is AFTER the watchdog restart: with the gateway still blocked, FailClose must RE-ENGAGE (traffic blocked again); then restore gateway access — traffic unblocks
+6. Restore gateway access — verify tunnel reconnects AND traffic unblocks WITHOUT a client restart
+7. Service crash edge case: crash is a deliberate fail-open (driver auto-teardown drops WFP blocking) — traffic flowing in the crash window is expected, NOT a failure. After watchdog restart with gateway still blocked, FailClose must re-engage (traffic blocked again); restore gateway — traffic unblocks
 8. (OPTIONAL — NPA-licensed tenants only; auto-detect via nsdiag -n, skip when NPA status is N/A, mirroring STRESS-03's NPA pattern) Test edge case: FailClose + NPA-only tunnel (ENG-1012026 pattern) — verify cert-pinned apps are also blocked</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>All non-exempt traffic blocked while FailClose is engaged (gateway unreachable). Traffic restored after gateway recovery WITHOUT a client restart. No permanent block state. Service crash is a deliberate FAIL-OPEN (driver auto-teardown): traffic flows during the crash window — this is expected, NOT a failure. After the watchdog restarts the service with the gateway still blocked, FailClose must re-engage and block again. Captive portal detection works (OPTIONAL — non-blocking until a captive-portal-capable environment exists). Cert-pinned apps blocked under FailClose + NPA-only tunnel (OPTIONAL — verified only on NPA-licensed tenants, auto-detected via nsdiag -n; skipped when N/A).</t>
+          <t>Traffic blocked while FailClose engaged. Traffic restored after gateway recovery WITHOUT a client restart. No permanent block. Crash-window fail-open is by design (expected, not a failure); FailClose must re-engage after watchdog restart while still fenced. (OPTIONAL, non-blocking) Captive portal detection. (OPTIONAL, NPA tenants only, auto-detect via nsdiag -n) Cert-pinned apps blocked under NPA-only tunnel.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: restore AOAC-02 (Hibernate S4 & Resume) into both copies
Mirrors nsclient_test_base 20ead5b. AOAC-02 existed only in the superseded
system_test_v3.xlsx snapshot; a full audit of v3/v4 against every remaining copy
showed it was the ONLY row missing from canonical (v4 contributes nothing, and
neither snapshot had a column non-empty there but empty in canonical).

Sourced from v3 rather than system_test_phase_1.xlsx, whose copy of the same row
has an empty Detailed Explanation -- v3 carries the full 452-char rationale.

Verified: exactly one AOAC-02 row per copy, all 9 columns populated.
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -4760,15 +4760,59 @@
       <c r="Z64" s="6" t="n"/>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="5">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
-      <c r="I65" s="6" t="n"/>
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>AOAC-02</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Hibernate (S4) &amp; Resume</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Power Management / Service Lifecycle</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Tests NSClient behavior across full hibernate (S4 — memory saved to disk, full power off) and resume. Unlike Modern Standby, S4 means ALL state is lost — network adapters reset, services see a cold-start-like event but with preserved process memory. Tests whether the service correctly re-detects network, re-establishes tunnel, and whether any in-memory state (tunnel state machine, config cache, GSLB selection) becomes stale or corrupt after resume.</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>1. Establish tunnel, verify traffic flowing
+2. Trigger hibernate (shutdown /h)
+3. Resume from hibernate
+4. Verify: stAgentSvc is running (should survive hibernate as service)
+5. Verify: tunnel reconnects — network detection fires on resume
+6. Verify: config is still valid (not expired during hibernate period)
+7. Verify: GSLB cache is refreshed (POP might have changed while hibernated)
+8. Test: hibernate for extended period (2+ hours) then resume — verify cert hasn't expired, config re-downloads
+9. Verify: FailClose handles the transition correctly (doesn't block during reconnect window)</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>Service survives hibernate. Tunnel reconnects within 30s of resume. Config re-validated. No stale GSLB state.</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>After hibernate: tunnel never reconnects, user has no security coverage. Or FailClose activates permanently because tunnel state is stale from pre-hibernate.</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Service lifecycle gaps (45% test gap rate in ch.03). Power event handling in stAgentSvc.cpp.</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Confluence Page - Windows System Test Plan</t>
+        </is>
+      </c>
       <c r="J65" s="6" t="n"/>
       <c r="K65" s="6" t="n"/>
       <c r="L65" s="6" t="n"/>

</xml_diff>

<commit_message>
spec: STRESS-07 step-8 refined per ENG-1012026 live repro (both copies)
Agent: git33-kimi-k3
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -743,12 +743,12 @@
 5. (OPTIONAL — requires a captive-portal-capable WiFi environment, not available on current lane VMs; non-blocking) Verify: captive portal detection triggers if connecting to new WiFi with portal
 6. Restore gateway access — verify tunnel reconnects AND traffic unblocks WITHOUT a client restart
 7. Service crash edge case: crash is a deliberate fail-open (driver auto-teardown drops WFP blocking) — traffic flowing in the crash window is expected, NOT a failure. After watchdog restart with gateway still blocked, FailClose must re-engage (traffic blocked again); restore gateway — traffic unblocks
-8. (OPTIONAL — NPA-licensed tenants only; auto-detect via nsdiag -n, skip when NPA status is N/A, mirroring STRESS-03's NPA pattern) Test edge case: FailClose + NPA-only tunnel (ENG-1012026 pattern) — verify cert-pinned apps are also blocked</t>
+8. (OPTIONAL — NPA-licensed tenants only; auto-detect via nsdiag -n, skip when NPA is not Connected) FailClose + NPA User Tunnel (ENG-1012026): with FailClose armed, block BOTH the CASB gateway and the NPA gateway -&gt; restart -&gt; FAIL_CLOSED. Verify: non-CPA traffic is blocked AND cert-pinned app flows (decrypt-action CPA, e.g. [tlstest]) are also blocked — expected evidence 'FailClosed flow dropped:: ... process: &lt;cpa proc&gt;' in nsdebuglog. Note: the ticket's claimed mechanism (NPA in m_tunnelIds) is source-disputed, but live repro on tenant 1347 (2026-07-30) shows the decrypt-action CPA bypasses FailClose via bypassAppMgr 'Bypassing connection ... to be decrypted' — the assertion documents the CORRECT behavior; a bypass is the bug signature</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Traffic blocked while FailClose engaged. Traffic restored after gateway recovery WITHOUT a client restart. No permanent block. Crash-window fail-open is by design (expected, not a failure); FailClose must re-engage after watchdog restart while still fenced. (OPTIONAL, non-blocking) Captive portal detection. (OPTIONAL, NPA tenants only, auto-detect via nsdiag -n) Cert-pinned apps blocked under NPA-only tunnel.</t>
+          <t>Traffic blocked while FailClose engaged. Traffic restored after gateway recovery WITHOUT a client restart. No permanent block. Crash-window fail-open is by design (expected, not a failure); FailClose must re-engage after watchdog restart while still fenced. (OPTIONAL, non-blocking) Captive portal detection. (OPTIONAL, NPA tenants only, auto-detect via nsdiag -n) Under FailClose + NPA User Tunnel with both gateways blocked: non-CPA traffic blocked AND cert-pinned apps blocked ('FailClosed flow dropped::' + process in log); a cert-pinned 'Bypassing connection' line while fenced = FAIL.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: STRESS-07 steps + pass criteria — final short form (both copies)
Agent: git33-kimi-k3
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -738,17 +738,17 @@
         <is>
           <t>1. Enable FailClose in client configuration
 2. Establish tunnel — verify normal traffic flows
-3. Simulate gateway unreachable (block gateway IP at firewall/hosts)
-4. Verify: all user traffic is blocked (cannot browse, cannot reach any external site)
-5. (OPTIONAL — requires a captive-portal-capable WiFi environment, not available on current lane VMs; non-blocking) Verify: captive portal detection triggers if connecting to new WiFi with portal
+3. Simulate gateway unreachable (block gateway IP at firewall)
+4. Verify: all user traffic is blocked
+5. (OPTIONAL, non-blocking — no captive-portal-capable env) Captive portal detection on new WiFi
 6. Restore gateway access — verify tunnel reconnects AND traffic unblocks WITHOUT a client restart
-7. Service crash edge case: crash is a deliberate fail-open (driver auto-teardown drops WFP blocking) — traffic flowing in the crash window is expected, NOT a failure. After watchdog restart with gateway still blocked, FailClose must re-engage (traffic blocked again); restore gateway — traffic unblocks
-8. (OPTIONAL — NPA-licensed tenants only; auto-detect via nsdiag -n, skip when NPA is not Connected) FailClose + NPA User Tunnel (ENG-1012026): with FailClose armed, block BOTH the CASB gateway and the NPA gateway -&gt; restart -&gt; FAIL_CLOSED. Verify: non-CPA traffic is blocked AND cert-pinned app flows (decrypt-action CPA, e.g. [tlstest]) are also blocked — expected evidence 'FailClosed flow dropped:: ... process: &lt;cpa proc&gt;' in nsdebuglog. Note: the ticket's claimed mechanism (NPA in m_tunnelIds) is source-disputed, but live repro on tenant 1347 (2026-07-30) shows the decrypt-action CPA bypasses FailClose via bypassAppMgr 'Bypassing connection ... to be decrypted' — the assertion documents the CORRECT behavior; a bypass is the bug signature</t>
+7. Service crash edge case: deliberate fail-open — traffic flowing in the crash window is expected, NOT a failure. After watchdog restart with gateway still blocked, FailClose must re-engage; restore gateway — traffic unblocks
+8. (OPTIONAL — NPA tenants only; auto-skip) FailClose + NPA-only tunnel: cert-pinned apps must also be blocked</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Traffic blocked while FailClose engaged. Traffic restored after gateway recovery WITHOUT a client restart. No permanent block. Crash-window fail-open is by design (expected, not a failure); FailClose must re-engage after watchdog restart while still fenced. (OPTIONAL, non-blocking) Captive portal detection. (OPTIONAL, NPA tenants only, auto-detect via nsdiag -n) Under FailClose + NPA User Tunnel with both gateways blocked: non-CPA traffic blocked AND cert-pinned apps blocked ('FailClosed flow dropped::' + process in log); a cert-pinned 'Bypassing connection' line while fenced = FAIL.</t>
+          <t>Traffic blocked while FailClose engaged. Traffic restored after gateway recovery WITHOUT a client restart. No permanent block. Crash-window fail-open is by design; FailClose must re-engage after watchdog restart while still fenced. (OPTIONAL, non-blocking) Captive portal detection. (OPTIONAL, NPA only) Cert-pinned apps blocked under FailClose + NPA-only tunnel.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: STRESS-13 steps + pass criteria — short form (both copies)
Agent: git33-kimi-k3
Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -2968,16 +2968,16 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>1. Configure cert-pinned exception for a specific app (e.g., Teams)
-2. Verify only that app's traffic bypasses tunnel
-3. Generate traffic from other apps
-4. Verify other apps still steered through tunnel
-5. Change steering config and verify cert-pinned exception still scoped correctly</t>
+          <t>1. Register tlstest.exe as a cert-pinned app with bypass action
+2. Generate traffic from tlstest.exe, another app, and a non-CPA control app to the same destinations — verify only tlstest bypasses the tunnel; the others stay steered
+3. Verify the exception does not broaden: no other app's traffic bypasses, to any destination
+4. Switch tlstest's action to decrypt
+5. Verify decryption takes effect for tlstest traffic; other apps stay steered</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Only cert-pinned app traffic bypasses; all other traffic remains steered; config change does not broaden exception scope</t>
+          <t>Only the cert-pinned app's traffic bypasses; all other traffic stays steered — no broadening of exception scope to other apps or domains. Switching the app action to decrypt takes effect, with decryption evidenced for the app's flows.</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">

</xml_diff>

<commit_message>
spec: add STEER-05 as a formal subset of STEER-01
test_steer_05_fast.py (merged via PR #412, win/mac split) validates STEER-01's
steps 1/5/6 in isolation via an HTTPS cert-issuer check, skipping the slow
long-lived-download steps. It had no spec row despite being a real, actively
maintained test case -- added one, cross-referencing STEER-01.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -4832,15 +4832,55 @@
       <c r="Z65" s="6" t="n"/>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="5">
-      <c r="A66" s="6" t="n"/>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
-      <c r="I66" s="6" t="n"/>
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>STEER-05</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Steering Rule Update Fast Verification (subset of STEER-01)</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Steering / Traffic Interception</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>Fast, isolated subset of STEER-01 (test_steer_05_fast.py, PR #412, merged 2026-08-26): validates only step 1 (client healthy, Cloud Apps traffic mode), step 5 (new connection steered after a rule change), and step 6 (still steered after the leak-grace period). Skips STEER-01's slow steps 2-4 (long-lived download through a rule change). Uses a dedicated HTTPS verify domain instead of an HTTP long-lived-download host: a TLS cert re-signed by the Netskope CA is authoritative proof the connection was steered -- more reliable than the 'Tunneling flow' debug-log marker alone, which is racy for short connections. Runs as separate Windows and Mac test functions (test_steer_05_fast_new_conn_steered / _mac), sharing one pyrobin.case ID with STEER-01 (same spec item, two automations).</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>1. Ensure client healthy: enrolled, tunnel CONNECTED; force traffic mode to Cloud Apps Only via the bound steering config if not already set (restored in teardown).
+2. Add a dedicated HTTPS verify domain to the steering (managed cloud apps) list; push and content-verify the domain actually landed in the client's nssteering.json (not just that the push API returned success).
+3. Flush DNS, then start a NEW connection (curl) to the verify domain.
+4. Verify the new connection is steered: check the debug-log 'Tunneling flow' marker first, then fall back to TLS cert issuer = Netskope CA. Retry up to 4 times with short backoff.
+5. Wait the leak-grace period, flush DNS, start another new connection, and re-verify it is still steered (no permanent bypass leak after the grace window).</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>New connection to the just-steered domain is steered promptly (debug-log marker or Netskope-CA cert issuer) within the retry window. After the leak-grace period, a fresh connection to the same domain is still steered -- no reversion to bypass.</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Same class of gap as STEER-01 but caught faster: a newly steering-added domain is not promptly enforced for new connections, or reverts to bypass after the grace window -- a security policy gap on always-on/frequently-reconnecting apps.</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Same as STEER-01: Ch. 09 (Traffic Interception), Ch. 05 (Steering Configuration). Fast subset isolating STEER-01's flaky steps 5/6 from its slow long-lived-download steps 2-4.</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>New - formal test case as of PR #412 (2026-08-26), split into windows/mac wrappers; subset of STEER-01 (test_steer_05_fast.py), intended to be merged back into test_steer_p0.py's full 7-step case once stable.</t>
+        </is>
+      </c>
       <c r="J66" s="6" t="n"/>
       <c r="K66" s="6" t="n"/>
       <c r="L66" s="6" t="n"/>

</xml_diff>

<commit_message>
spec: add STRESS-02-MAC row for the per-protocol flood face (mac)
The STRESS-02 row only describes the sustained-HTTPS-bandwidth face.
The per-protocol face (DNS/UDP/FTP/SFTP simultaneously) that the mac
automation now covers had no spec row at all, so add one instead of
overloading STRESS-02 with two different loads.

All three canonical copies written via system_test_xlsx.py --both.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -4900,15 +4900,55 @@
       <c r="Z66" s="6" t="n"/>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="5">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="6" t="n"/>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="6" t="n"/>
-      <c r="H67" s="6" t="n"/>
-      <c r="I67" s="6" t="n"/>
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>STRESS-02-MAC</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Per-Protocol Traffic Flood (DNS/UDP/FTP/SFTP) - mac</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Tunneling / Stress</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Per-protocol face of STRESS-02: drives DNS, UDP, FTP and SFTP volume SIMULTANEOUSLY, instead of the sustained-HTTPS-bandwidth face the STRESS-02 row already covers, and gates client survival under it (tunnel stays connected, steering binding unchanged, client processes alive, bounded memory growth). This is the automation of what QA runs by hand on Macs every release with the local stress_test tool. Mac automation = test_stress_02_protocol_flood_mac, driving a stdlib-only VM-side generator (stock mac python3, no pip packages; the SFTP leg shells out to the stock /usr/bin/sftp client). Shares the SYS-STRESS-02 case ID with the bandwidth face - same spec item, two automations. Deliberately NOT covered: MTU 1300-vs-9000 variation and packet-loss injection (needs a network conditioner; only the UDP payload size is configurable), and GRE/IPsec flooding (cannot be emitted from userland python).</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>1. Client daemon running and tunnel CONNECTED; capture the bound steering config name and the client memory baseline
+2. Start a simultaneous per-protocol flood from the mac for &gt;=4 min: DNS random-subdomain queries, UDP datagrams, FTP uploads, SFTP uploads
+3. Poll the tunnel for the whole load window - it must never disconnect
+4. Read the per-protocol counters: every enabled protocol must show real volume (missing counters = harness failure, not a product result; all file transfers failing = environment failure)
+5. Verify the bound steering config is unchanged, the tunnel is still connected, client health processes are alive, and client memory growth is under the ceiling</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>Zero tunnel disconnects across the flood window; every enabled protocol records non-zero volume (FTP/SFTP additionally record non-zero SUCCESSFUL uploads); bound steering config unchanged; client health processes alive; client memory growth &lt;50MB over the window. Consistent across all repetitions (--iterations).</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Non-HTTP protocol volume destabilises the client: the tunnel drops or the steering binding changes under load, or memory grows unbounded - leaving traffic unprotected on exactly the protocols customers saturate in production, and on the platform where this load is currently only ever checked by hand.</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Per-release manual mac protocol-flood runs: ENG-914348~352 (R136), ENG-950122 series (R137). Same spec-row family as STRESS-02 (EIMF-237/EIMF-344 slow downloads, IMF-1325 HAProxy CPU).</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>NSClient Reliability Test Plan - STRESS-02 per-protocol face (the STRESS-02 row keeps the sustained-bandwidth face). Mac automation added 2026-09-04 (PR 442, ns-klin); ported from the per-protocol half of the local stress_test tool.</t>
+        </is>
+      </c>
       <c r="J67" s="6" t="n"/>
       <c r="K67" s="6" t="n"/>
       <c r="L67" s="6" t="n"/>

</xml_diff>

<commit_message>
spec(SystemTest): renumber mac per-protocol flood row from STRESS-02-MAC to STRESS-27
STRESS-09 was proposed for this new row but is already occupied by an
unrelated, implemented case (FailClose x DNS security x steering mode
transitions). STRESS-27 is the next genuinely free ID (13/19/23 are also
already spoken for or deliberately-skipped gaps). Drops the "shares the
SYS-STRESS-02 case ID" framing since this is now its own independent case.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/regression/system_test_new.xlsx
+++ b/regression/system_test_new.xlsx
@@ -4902,7 +4902,7 @@
     <row r="67" ht="15.75" customHeight="1" s="5">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>STRESS-02-MAC</t>
+          <t>STRESS-27</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Per-protocol face of STRESS-02: drives DNS, UDP, FTP and SFTP volume SIMULTANEOUSLY, instead of the sustained-HTTPS-bandwidth face the STRESS-02 row already covers, and gates client survival under it (tunnel stays connected, steering binding unchanged, client processes alive, bounded memory growth). This is the automation of what QA runs by hand on Macs every release with the local stress_test tool. Mac automation = test_stress_02_protocol_flood_mac, driving a stdlib-only VM-side generator (stock mac python3, no pip packages; the SFTP leg shells out to the stock /usr/bin/sftp client). Shares the SYS-STRESS-02 case ID with the bandwidth face - same spec item, two automations. Deliberately NOT covered: MTU 1300-vs-9000 variation and packet-loss injection (needs a network conditioner; only the UDP payload size is configurable), and GRE/IPsec flooding (cannot be emitted from userland python).</t>
+          <t>Per-protocol face of the mac stress family: drives DNS, UDP, FTP and SFTP volume SIMULTANEOUSLY, instead of the sustained-HTTPS-bandwidth face STRESS-02 covers, and gates client survival under it (tunnel stays connected, steering binding unchanged, client processes alive, bounded memory growth). This is the automation of what QA runs by hand on Macs every release with the local stress_test tool. Mac automation = test_stress_02_protocol_flood_mac, driving a stdlib-only VM-side generator (stock mac python3, no pip packages; the SFTP leg shells out to the stock /usr/bin/sftp client). Independent case ID SYS-STRESS-27 (previously staged under a shared STRESS-02 ID; split out to avoid colliding with STRESS-09, which is unrelated). Deliberately NOT covered: MTU 1300-vs-9000 variation and packet-loss injection (needs a network conditioner; only the UDP payload size is configurable), and GRE/IPsec flooding (cannot be emitted from userland python).</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>NSClient Reliability Test Plan - STRESS-02 per-protocol face (the STRESS-02 row keeps the sustained-bandwidth face). Mac automation added 2026-09-04 (PR 442, ns-klin); ported from the per-protocol half of the local stress_test tool.</t>
+          <t>NSClient Reliability Test Plan - mac per-protocol flood face, independent case ID SYS-STRESS-27 (STRESS-02 keeps the sustained-bandwidth face). Mac automation added 2026-09-04 (PR 442, ns-klin); ported from the per-protocol half of the local stress_test tool.</t>
         </is>
       </c>
       <c r="J67" s="6" t="n"/>

</xml_diff>